<commit_message>
Add domain-behaviour analysis track; exclusion claims in domain reference; archive dead ends
- domain-behaviour/: Domain_Behaviour.ipynb re-derives fan-out, decomposition axes and
  scale/units per domain from COSMoS; tests the Consumer_Exclusions claims; publishes
  docs/analyses/domain-behaviour.html, linked from a new Analyses section on the landing page
- SDTM_Domain_Metadata: Consumer_Exclusions sheet; Findings consumers read exclusions from it
- IS and GF exclusion reasons restated (binding agent, test detail); all claims hold at COSMoS 2026-07-14
- docs/Data_Flow.md: release run order for SDTM CT and COSMoS releases
- Archived: NCIt-comparison notebooks (read retired flatten), evs_root_gap_coverage, Top_Level_Summary

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ndgbpomxbp7qzdpv1ucjv
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domains" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelist_Overrides" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrument_Domain_Rules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumer_Exclusions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Domains'!$A$1:$G$57</definedName>
@@ -469,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -640,264 +641,353 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Consumer_Exclusions</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Domains a Findings consumer leaves out of its scope, each reason stated as testable claims (5 rows)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>COLUMN DESCRIPTIONS</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Two-letter SDTM domain abbreviation (RELREC/RELSPEC for relationship datasets)</t>
-        </is>
-      </c>
+      <c r="B21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Domain_Name</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Full domain name from SDTMIG v3.4; for domains added from CT, the C66734 name</t>
+          <t>Two-letter SDTM domain abbreviation (RELREC/RELSPEC for relationship datasets)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Observation_Class</t>
+          <t>Domain_Name</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design, Relationship</t>
+          <t>Full domain name from SDTMIG v3.4; for domains added from CT, the C66734 name</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SDTMIG_Section</t>
+          <t>Observation_Class</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Section number in SDTMIG v3.4 where the domain is specified (empty for domains added from CT)</t>
+          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design, Relationship</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Has_Test_Codes</t>
+          <t>SDTMIG_Section</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
+          <t>Section number in SDTMIG v3.4 where the domain is specified (empty for domains added from CT)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Specimen_Based</t>
+          <t>Has_Test_Codes</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is specimen-based per SDTMIG v3.4 Section 6.3.5 (Yes/No)</t>
+          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Specimen_Based</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is a subject-level measurement domain (Yes/No). Measurement_Findings takes its scope from this flag, minus exclusions named in the notebook.</t>
+          <t>Whether the domain is specimen-based per SDTMIG v3.4 Section 6.3.5 (Yes/No)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain is a subject-level measurement domain (Yes/No). Measurement_Findings takes its scope from this flag, minus exclusions named in the notebook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Brief notes on domain status or version history</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-      <c r="B29" s="2" t="n"/>
-    </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>CODELIST_OVERRIDES COLUMNS</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>CT_Display_Name</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>The codelist display name from NCI EVS (after stripping " Test Code")</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>CT_Display_Name</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Target SDTM domain abbreviation (empty for Cross-domain)</t>
+          <t>The codelist display name from NCI EVS (after stripping " Test Code")</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Override_Type</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Naming (label mismatch), Subset (body-system sub-codelist), or Cross-domain (test code codelist shared by several domains; Domain empty)</t>
+          <t>Target SDTM domain abbreviation (empty for Cross-domain)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>Override_Type</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Naming (label mismatch), Subset (body-system sub-codelist), or Cross-domain (test code codelist shared by several domains; Domain empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Description of the mismatch</t>
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>INSTRUMENT_DOMAIN_RULES COLUMNS</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Keyword</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Instrument class. Matched first as the prefix "CDISC &lt;Keyword&gt; " of the codelist NCI Preferred Term, then as a substring of the codelist display name</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Target SDTM domain abbreviation</t>
+          <t>Instrument class. Matched first as the prefix "CDISC &lt;Keyword&gt; " of the codelist NCI Preferred Term, then as a substring of the codelist display name</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Target SDTM domain abbreviation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Description and examples of instrument types in this category</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>KNOWN LIMITATIONS</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n"/>
-    </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n"/>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>CONSUMER_EXCLUSIONS COLUMNS</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="n"/>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Findings consumer notebook that reads the row (Specimen_Findings, Measurement_Findings, Instrument_Findings)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SDTM v3.0 is under review and may add or change domains.</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n"/>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Domain excluded from that consumer's scope</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n"/>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Identifier of one testable claim behind the exclusion</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>What the published COSMoS content must show for the exclusion reason to hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Machine form of the claim, evaluated by domain-behaviour/notebooks/Domain_Behaviour.ipynb: no_fanout, no_axis, not_axis:&lt;axis&gt;, axis_all:&lt;axis&gt;, not_primary:&lt;axis&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>The exclusion reason as recorded in the consumer notebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>KNOWN LIMITATIONS</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>That requires CDISC membership access to the SDTM v2.0 Excel files.</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>SDTM v3.0 is under review and may add or change domains.</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t>SDTMIG section numbers are reconstructed from public sources — verify against the IG.</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3859,4 +3949,218 @@
   <autoFilter ref="A1:C4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Specimen_Findings</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>IS-1</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Every BC that fans out differs by binding agent</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>axis_all:binding agent</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Target-driven, not specimen-driven: the DSSs of one BC differ by binding agent (BDAGNT), the target. The March 2026 analysis found the target only in the DS code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Specimen_Findings</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>IS-2</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Specimen is not the primary axis</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>not_primary:specimen</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Target-driven, not specimen-driven: the DSSs of one BC differ by binding agent (BDAGNT), the target. The March 2026 analysis found the target only in the DS code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Specimen_Findings</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>GF</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>GF-1</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Every BC that fans out differs by test detail</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>axis_all:test detail</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Test-detail-driven, not specimen-driven: the DSSs of one BC differ by test detail (TSTDTL). The March 2026 analysis recorded it as scale-driven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Specimen_Findings</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>GF</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>GF-2</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Specimen is not the primary axis</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>not_primary:specimen</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Test-detail-driven, not specimen-driven: the DSSs of one BC differ by test detail (TSTDTL). The March 2026 analysis recorded it as scale-driven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Specimen_Findings</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>UR-1</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No BC has more than one DSS</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>no_fanout</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Zero decomposition despite Specimen_Based metadata flag.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Variable_Meaning reviewed: 20 positions accepted, ISTSTDTL and VSPOS held
Held rows carry the reason in Basis_Note. Observables_Direction: the 2026-10-06 reading is labelled as before Phase 1; where it differs, Variable_Meaning holds.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01MfbDja99K4rW2RjUAKiaQk
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -839,7 +839,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
@@ -883,7 +882,6 @@
         </is>
       </c>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
@@ -963,7 +961,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
@@ -1055,7 +1052,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
@@ -4368,7 +4364,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4401,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4438,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4475,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4512,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4549,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4590,7 +4586,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4618,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>COSMoS only: predicate SPECIFIES, "further describes the test in", codelist ISFTSDTL; DEC label not stated on all DSSs. Fan-out and key agree (Key_Compare). IS DSSs pin no LOINC codes.</t>
+          <t>COSMoS only: predicate SPECIFIES, "further describes the test in", codelist ISFTSDTL; DEC label not stated on all DSSs. Fan-out and key agree (Key_Compare). IS DSSs pin no LOINC codes. Held 2026-10-08: DEC label not stated on all DSSs.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -4664,7 +4660,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4697,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4738,7 +4734,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4775,7 +4771,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4785,7 +4781,6 @@
           <t>Key_Compare</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>scale</t>
@@ -4808,7 +4803,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4840,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4882,7 +4877,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4914,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4951,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4988,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5025,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -5062,7 +5057,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable.</t>
+          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable. Held 2026-10-08: LOINC has position-free and position-qualified codes side by side; to be backed by a cell before the row is accepted.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5104,7 +5099,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5136,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable_Meaning: notes from the SDTMIG v3.4 Assumptions
Basis notes cite IG_Assumptions (LB 8, GF 8, MB 1, MI 2, IS 7, RS, TR 1-2)
for LBSPEC, LBMETHOD, GFMETHOD, GFANMETH, MBTSTDTL, ISBDAGNT, RSCAT,
VSPOS, RSEVAL, MITSTDTL, TRGRPID and LBFAST. TRGRPID accepted;
MITSTDTL stays proposed; LBFAST stays open (LB 8: an aspect of the
test when the LOINC code distinguishes it - carried into Phase 2).

Observables_Phase1: the IG Assumptions as a source, quoted in the
agree, disagree and silent sections.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MfbDja99K4rW2RjUAKiaQk
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -4359,7 +4359,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>COSMoS: predicate IS_SPECIMEN_TESTED_IN, "is the specimen tested in", codelist SPECTYPE. Fan-out axis specimen and key part system agree (Key_Compare). LOINC system agrees (LOINC_Compare); the exceptions are COSMoS pin errors reported by COSMoS_Observable_LOINC_Check. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them.</t>
+          <t>COSMoS: predicate IS_SPECIMEN_TESTED_IN, "is the specimen tested in", codelist SPECTYPE. Fan-out axis specimen and key part system agree (Key_Compare). LOINC system agrees (LOINC_Compare); the exceptions are COSMoS pin errors reported by COSMoS_Observable_LOINC_Check. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>COSMoS: predicate SPECIFIES, "is the method for the test in", DEC Test Method, codelist METHOD. Fan-out axis method and key part method agree (Key_Compare). LOINC method agrees where COSMoS separates by method (LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them.</t>
+          <t>COSMoS: predicate SPECIFIES, "is the method for the test in", DEC Test Method, codelist METHOD. Fan-out axis method and key part method agree (Key_Compare). LOINC method agrees where COSMoS separates by method (LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>COSMoS only: predicate SPECIFIES, DEC Test Method, codelist METHOD. Fan-out and key agree (Key_Compare). GF DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them.</t>
+          <t>COSMoS only: predicate SPECIFIES, DEC Test Method, codelist METHOD. Fan-out and key agree (Key_Compare). GF DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 GF Assumption 8 (IG_Assumptions): 'GFMETHOD lists wet lab techniques …; methods related to specimen processing or reagents are not represented in GFMETHOD.'</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate SPECIFIES, "further describes the test in", DEC Measurement, Test or Examination Detail, codelist MBFTSDTL. Fan-out and key agree (Key_Compare). LOINC not read for MB (not in LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD.</t>
+          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate SPECIFIES, "further describes the test in", DEC Measurement, Test or Examination Detail, codelist MBFTSDTL. Fan-out and key agree (Key_Compare). LOINC not read for MB (not in LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 MB Assumption 1 (IG_Assumptions): 'DETECTION' for tests that identify an organism; for a characteristic, 'the name of the characteristic being described (e.g., COLONY COUNT, VIRAL LOAD)'.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>COSMoS: SPECIFIES, "further describes the test in", codelist MIFTSDTL. SDTM v2.0: Variable Qualifier of --TESTCD, like the other --TSTDTL rows. SDTMIG v3.4 MI: Record Qualifier. Rule, for now: the Model's Variables Qualified and the sibling --TSTDTL rows hold over the IG role.</t>
+          <t>COSMoS: SPECIFIES, "further describes the test in", codelist MIFTSDTL. SDTM v2.0: Variable Qualifier of --TESTCD, like the other --TSTDTL rows. SDTMIG v3.4 MI: Record Qualifier. Rule, for now: the Model's Variables Qualified and the sibling --TSTDTL rows hold over the IG role. SDTMIG v3.4 MI Assumption 2 (IG_Assumptions): 'MITSTDTL further qualifies the record' — the IG prose matches its own Record Qualifier role.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate IS_ATTRIBUTE_FOR, "is the substance bound to the analyte in", codelists ISBDAGT and MICROORG. Fan-out axis binding agent and key part component agree (Key_Compare). IS DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD.</t>
+          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate IS_ATTRIBUTE_FOR, "is the substance bound to the analyte in", codelists ISBDAGT and MICROORG. Fan-out axis binding agent and key part component agree (Key_Compare). IS DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 IS Assumption 7 (IG_Assumptions): two codelists (MICROORG, ISBDAGT); the CT Rules for Immunogenicity Tests say which to use.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>COSMoS: predicate SPECIFIES, "is the method of secondary analysis of results in", DEC Analysis Method, codelist GFANMET. Not DEC Test Method, so not the test method; the key reads --METHOD only (Key_Compare: method, fan-out only). No source says whether the analysis method is part of the observable. SDTMIG v3.4: Record Qualifier, 'the method of secondary processing performed by the dry lab to yield the result'.</t>
+          <t>COSMoS: predicate SPECIFIES, "is the method of secondary analysis of results in", DEC Analysis Method, codelist GFANMET. Not DEC Test Method, so not the test method; the key reads --METHOD only (Key_Compare: method, fan-out only). No source says whether the analysis method is part of the observable. SDTMIG v3.4: Record Qualifier, 'the method of secondary processing performed by the dry lab to yield the result'. SDTMIG v3.4 GF Assumption 8 (IG_Assumptions) confines GFMETHOD to wet lab techniques; the IG note puts GFANMETH in the dry lab (secondary processing).</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>COSMoS: predicate GROUPS, "groups values in", the same as LBCAT. SDTM CT codelist ONCRSCAT, Category of Oncology Response Assessment: the response criteria. Not in the key. No source says whether category changes the observation. SDTM v2.0 and SDTMIG v3.4: Grouping Qualifier; the IG notes that the RSCAT codelist depends on whether the records are oncology response criteria or another clinical classification.</t>
+          <t>COSMoS: predicate GROUPS, "groups values in", the same as LBCAT. SDTM CT codelist ONCRSCAT, Category of Oncology Response Assessment: the response criteria. Not in the key. No source says whether category changes the observation. SDTM v2.0 and SDTMIG v3.4: Grouping Qualifier; the IG notes that the RSCAT codelist depends on whether the records are oncology response criteria or another clinical classification. SDTMIG v3.4 RS Assumptions (IG_Assumptions; disease response 1, 6, 9; clinical classifications 2): RSCAT 'is used to group a set of assessments based on' a disease response criterion or a clinical classification; 'UNSPECIFIED' when the criteria are unknown.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -5020,12 +5020,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SDTM v2.0 and SDTMIG v3.4: Identifier, "used to link together a block of related records within a subject in a domain". COSMoS states nothing (no predicate, no codelist). One source states it, none contradicts.</t>
+          <t>SDTM v2.0 and SDTMIG v3.4: Identifier, "used to link together a block of related records within a subject in a domain". COSMoS states nothing (no predicate, no codelist). One source states it, none contradicts. SDTMIG v3.4 TR Assumptions 1 and 2 (IG_Assumptions): --GRPID 'may be used for other purposes, per the SDTM', so TR/TU links use --LNKID/--LNKGRP instead.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>accepted</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable. LOINC (Subject_State in COSMoS_Observable_LOINC_Check): position-free and position-qualified codes side by side (^sitting, ^standing, ^supine); COSMoS assigns VSPOS on no DSS. LOINC offers position as a refinement, not as a requirement. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers.</t>
+          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable. LOINC (Subject_State in COSMoS_Observable_LOINC_Check): position-free and position-qualified codes side by side (^sitting, ^standing, ^supine); COSMoS assigns VSPOS on no DSS. LOINC offers position as a refinement, not as a requirement. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. The SDTMIG v3.4 VS Assumptions do not discuss VSPOS; LB Assumption 8 (IG_Assumptions) names LBPOS (in LB) among the LOINC-associated aspects of a test.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>COSMoS assigns RSEVAL = INVESTIGATOR on some DSSs, value list only on others (Rater_COSMoS_EVAL); SDTM CT codelist EVAL. A rater is also stated in NCIt definition prose (Rater_Evidence). No source ties the rater to the instrument as a property.</t>
+          <t>COSMoS assigns RSEVAL = INVESTIGATOR on some DSSs, value list only on others (Rater_COSMoS_EVAL); SDTM CT codelist EVAL. A rater is also stated in NCIt definition prose (Rater_Evidence). No source ties the rater to the instrument as a property. SDTMIG v3.4 RS disease response Assumption 7 (IG_Assumptions): RSEVALID with RSEVAL gives detail of who provides the assessment.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>COSMoS: LBFAST is a value list (N;Y), never assigned, so it never separates sibling DSSs and is not in Variable_Evidence. LOINC (Subject_State): fasting-free and fasting-qualified glucose codes side by side (component Glucose^post CFst, class CHAL). LOINC offers fasting as a refinement, not as a requirement; no source says whether fasting is part of the observable. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers.</t>
+          <t>COSMoS: LBFAST is a value list (N;Y), never assigned, so it never separates sibling DSSs and is not in Variable_Evidence. LOINC (Subject_State): fasting-free and fasting-qualified glucose codes side by side (component Glucose^post CFst, class CHAL). LOINC offers fasting as a refinement, not as a requirement; no source says whether fasting is part of the observable. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): LBFAST is among 'the aspects of a test that are associated with a LOINC code', 'only required to be populated when necessary to provide a semantically meaningful distinction between records with different LBLOINC values'. COSMoS, LOINC and the IG agree that subject state is an optional refinement; none says it is always or never part of the observable (decided 2026-10-08: open, the conditional reading carried into Phase 2).</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">

</xml_diff>

<commit_message>
Domain_Behaviour: Interpretation_Context; three proposed Variable_Meaning rows
Domain_Behaviour section 4i (before 4f, which reads it): new sheet
Interpretation_Context, one row per generic variable x domain for every
SDTM v2.0 Record Qualifier, Variable Qualifier and Timing variable, with the
SDTMIG v3.4 Core and codelist and how COSMoS uses it (absent, never
assigned, always assigned, mixed). What the record carries beside a value so
it can be read; the operational side of a study is outside. Key measures added.

Variable_Meaning: QSEVINTX, RSEVINTX, RSEVLINT as proposed, Position open,
basis standards silent - COSMoS always assigns the evaluation interval where
present; candidate for the instrument observable. Key_Source
Interpretation_Context accepted by the 4f check. Instrument_Findings
Axis_Meaning shows the three rows.
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -681,7 +681,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Our position on what a variable or axis means for the observable, Findings only, each with a stated basis (23 rows)</t>
+          <t>Our position on what a variable or axis means for the observable, Findings only, each with a stated basis (26 rows)</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Sheet of domain-behaviour/interim/Domain_Behaviour.xlsx the key must exist in: Variable_Evidence (Domain + variable), Key_Compare (axis; Domain empty), Rater_COSMoS_EVAL (variable_name); or LOINC_Subject_State: sheet Subject_State of cosmos-bc-dss/reports/COSMoS_Observable_LOINC_Check.xlsx (state_variable)</t>
+          <t>Sheet of domain-behaviour/interim/Domain_Behaviour.xlsx the key must exist in: Variable_Evidence (Domain + variable), Key_Compare (axis; Domain empty), Rater_COSMoS_EVAL (variable_name), Interpretation_Context (Domain + variable, with COSMoS content); or LOINC_Subject_State: sheet Subject_State of cosmos-bc-dss/reports/COSMoS_Observable_LOINC_Check.xlsx (state_variable)</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6002,6 +6002,117 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Interpretation_Context</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>QS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>QSEVINTX</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>standards silent, open</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Interpretation_Context: COSMoS_Use = always assigned in QS. SDTM v2.0 role Timing; SDTMIG v3.4 Core Perm. No source states whether the evaluation interval is part of what is observed or only context for reading the result. COSMoS fixing it on every DSS that carries it is consistent with the first. Candidate for the instrument observable.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Interpretation_Context</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RSEVINTX</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>standards silent, open</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Interpretation_Context: COSMoS_Use = always assigned in RS. SDTM v2.0 role Timing; SDTMIG v3.4 Core Perm. No source states whether the evaluation interval is part of what is observed or only context for reading the result. COSMoS fixing it on every DSS that carries it is consistent with the first. Candidate for the instrument observable.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Interpretation_Context</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RSEVLINT</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>standards silent, open</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Interpretation_Context: COSMoS_Use = always assigned in RS. SDTM v2.0 role Timing; SDTMIG v3.4 Core Perm. No source states whether the evaluation interval is part of what is observed or only context for reading the result. COSMoS fixing it on every DSS that carries it is consistent with the first. Candidate for the instrument observable.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ReadMe: common header, one sheet name, pinned reference versions
Every machine_actionable xlsx now has a ReadMe sheet (was README in four)
that starts with PURPOSE, SCOPE, SOURCE VERSIONS, KNOWN GAPS, SHEETS.
Versions come from the new Reference_Versions.json at the repo root; the
notebooks that read COSMoS stop when the pin differs from the newest
package_date in DSS_View. SDTM_Domain_Metadata edited by hand (no
notebook). Two stale texts corrected: the UNMATCHED '28% gap' in
Instrument_Findings (now 0) and the pointer to the retired sdtm-findings
track in SDTM_Instrument_Test_Identity. CLAUDE.md: pin file, rule 5.
Data sheets unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzSyuaqVq1B4PFnRpWB
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domains" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codelist_Overrides" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrument_Domain_Rules" sheetId="4" state="visible" r:id="rId4"/>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -487,13 +487,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>PROVENANCE</t>
+          <t>PURPOSE</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -501,87 +501,62 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>SDTMIG v3.4 variable table and table of contents (downloaded with a cdisc.org sign-in; checked 2026-10-12); SDTM CT SDTM Domain Abbreviation codelist C66734 for domains not in SDTMIG v3.4</t>
-        </is>
-      </c>
+          <t>Reference data for programmatic use by notebooks and other tracks.</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SDTM Model</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>v2.0</t>
-        </is>
-      </c>
+          <t>Contains factual properties of SDTM domains from SDTMIG v3.4 and SDTM CT.</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SDTMIG</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>v3.4 (2021, current as of March 2026)</t>
-        </is>
-      </c>
+          <t>Changes when a new SDTMIG version is published, or when SDTM CT brings test codes for a domain not yet listed (sdtm-findings-graph/notebooks/Scope_Check.ipynb).</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Created</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Variable_Meaning is the exception: our position, not a published fact, with the basis stated per row.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Repository</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>https://github.com/kerfors/cdisc-for-ai</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SCOPE</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>PURPOSE</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>All SDTMIG v3.4 domains of observations, Trial Design and Special-Purpose, plus the domains SDTM CT C66734 lists that are not in SDTMIG v3.4 (Notes say which). Datasets that are not domains of observations are in Non_Observation_Datasets.</t>
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Reference data for programmatic use by notebooks and other tracks.</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="n"/>
       <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Contains factual properties of SDTM domains from SDTMIG v3.4 and SDTM CT.</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>SOURCE VERSIONS</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -589,110 +564,119 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Changes when a new SDTMIG version is published, or when SDTM CT brings test codes for a domain not yet listed (sdtm-findings-graph/notebooks/Scope_Check.ipynb).</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n"/>
+          <t>SDTM CT</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 (pinned in Reference_Versions.json at the repo root; written here by hand, this file has no notebook)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Variable_Meaning is the exception: our position, not a published fact, with the basis stated per row.</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>COSMoS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14 (pinned; not read by this file)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SDTMIG v3.4 variable table and table of contents (downloaded with a cdisc.org sign-in; checked 2026-10-12); SDTM CT SDTM Domain Abbreviation codelist C66734 for domains not in SDTMIG v3.4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>SHEETS</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SDTM Model</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>v2.0</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Domains</t>
+          <t>SDTMIG</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>One row per SDTM domain: SDTMIG v3.4, plus domains added from SDTM CT C66734 (see Notes) (66 rows)</t>
+          <t>v3.4 (2021, current as of March 2026)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Codelist_Overrides</t>
+          <t>Created</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CT display names that do not match Domain_Name directly (7 rows)</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Instrument_Domain_Rules</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Keyword-to-domain mapping for non-extensible instrument codelists (3 rows)</t>
+          <t>https://github.com/kerfors/cdisc-for-ai</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Non_Observation_Datasets</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>SDTMIG v3.4 datasets that are not domains of observations, each with the reason (5 rows)</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Consumer_Exclusions</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Domains a Findings consumer leaves out of its scope, each reason stated as testable claims (4 rows)</t>
-        </is>
-      </c>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>KNOWN GAPS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Variable_Meaning</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Our position on what a variable or axis means for the observable, Findings only, each with a stated basis (26 rows)</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>CDISC publishes it as the SDTM v2.0 and SDTMIG v3.4 variable tables (sign-in at cdisc.org). Local copies sit in sdtm-domain-reference/downloads/ (gitignored); domain-behaviour reads them.</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>COLUMN DESCRIPTIONS</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>SDTM v3.0 is under review and may add or change domains.</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -700,291 +684,291 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Two-letter SDTM domain abbreviation</t>
-        </is>
-      </c>
+          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Domain_Name</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Domain name used to match SDTM CT codelist names (sdtm-test-codes/notebooks/SDTM_CT_Extract.ipynb); the SDTMIG v3.4 name for most domains, the C66734 name for domains added from CT. IG_Name has the IG name.</t>
-        </is>
-      </c>
+          <t>SDTMIG_Section, IG_Name, IG_Class, Has_Test_Codes and Specimen_Based, and the Non_Observation_Datasets sheet, are checked against SDTMIG v3.4 by sdtm-findings-graph/notebooks/Scope_Check.ipynb (section 5).</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Observation_Class</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design. FA and SR are Findings here (the consumers filter on it); IG_Class has Findings About.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>SDTMIG_Section</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Section number in the SDTMIG v3.4 table of contents (empty for domains added from CT). MB, MS (6.3.5.7) and PC, PP (6.3.5.9) are listed only under a group heading.</t>
-        </is>
-      </c>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>SHEETS</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Has_Test_Codes</t>
+          <t>Domains</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
+          <t>One row per SDTM domain: SDTMIG v3.4, plus domains added from SDTM CT C66734 (see Notes) (66 rows)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Specimen_Based</t>
+          <t>Codelist_Overrides</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is specimen-based: listed under SDTMIG v3.4 Section 6.3.5 Specimen-based Findings Domains (Yes/No)</t>
+          <t>CT display names that do not match Domain_Name directly (7 rows)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Instrument_Domain_Rules</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Whether the domain is a subject-level measurement domain (Yes/No). Measurement_Findings takes its scope from this flag, minus exclusions named in the notebook.</t>
+          <t>Keyword-to-domain mapping for non-extensible instrument codelists (3 rows)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Non_Observation_Datasets</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Brief notes on domain status or version history</t>
+          <t>SDTMIG v3.4 datasets that are not domains of observations, each with the reason (5 rows)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>IG_Name</t>
+          <t>Consumer_Exclusions</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Domain name in the SDTMIG v3.4 table of contents (the sheet name for MB, MS, PC, PP); empty for domains added from CT</t>
+          <t>Domains a Findings consumer leaves out of its scope, each reason stated as testable claims (4 rows)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>IG_Class</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Class in the SDTMIG v3.4 variable table; empty for domains added from CT</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Variable_Meaning</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Our position on what a variable or axis means for the observable, Findings only, each with a stated basis (26 rows)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="n"/>
       <c r="B35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>CODELIST_OVERRIDES COLUMNS</t>
-        </is>
-      </c>
+          <t>COLUMN DESCRIPTIONS</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CT_Display_Name</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>The codelist display name from NCI EVS (after stripping " Test Code")</t>
+          <t>Two-letter SDTM domain abbreviation</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Domain_Name</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Target SDTM domain abbreviation (empty for Cross-domain)</t>
+          <t>Domain name used to match SDTM CT codelist names (sdtm-test-codes/notebooks/SDTM_CT_Extract.ipynb); the SDTMIG v3.4 name for most domains, the C66734 name for domains added from CT. IG_Name has the IG name.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Override_Type</t>
+          <t>Observation_Class</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Naming (label mismatch), Subset (body-system sub-codelist), or Cross-domain (test code codelist shared by several domains; Domain empty)</t>
+          <t>SDTM observation class: Findings, Events, Interventions, Special-Purpose, Trial Design. FA and SR are Findings here (the consumers filter on it); IG_Class has Findings About.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>SDTMIG_Section</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Description of the mismatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="41"/>
+          <t>Section number in the SDTMIG v3.4 table of contents (empty for domains added from CT). MB, MS (6.3.5.7) and PC, PP (6.3.5.9) are listed only under a group heading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Has_Test_Codes</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain uses --TESTCD/--TEST variables (Yes/No)</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>INSTRUMENT_DOMAIN_RULES COLUMNS</t>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Specimen_Based</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Whether the domain is specimen-based: listed under SDTMIG v3.4 Section 6.3.5 Specimen-based Findings Domains (Yes/No)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Measurement</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Instrument class. Matched first as the prefix "CDISC &lt;Keyword&gt; " of the codelist NCI Preferred Term, then as a substring of the codelist display name</t>
+          <t>Whether the domain is a subject-level measurement domain (Yes/No). Measurement_Findings takes its scope from this flag, minus exclusions named in the notebook.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Target SDTM domain abbreviation</t>
+          <t>Brief notes on domain status or version history</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>IG_Name</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Description and examples of instrument types in this category</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
+          <t>Domain name in the SDTMIG v3.4 table of contents (the sheet name for MB, MS, PC, PP); empty for domains added from CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>IG_Class</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Class in the SDTMIG v3.4 variable table; empty for domains added from CT</t>
+        </is>
+      </c>
+    </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>NON_OBSERVATION_DATASETS COLUMNS</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Dataset</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>SDTMIG v3.4 dataset name</t>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>CODELIST_OVERRIDES COLUMNS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IG_Name</t>
+          <t>CT_Display_Name</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Name in the SDTMIG v3.4 table of contents (8.4.1 Supplemental Qualifiers (SUPP--) for SUPPQUAL)</t>
+          <t>The codelist display name from NCI EVS (after stripping " Test Code")</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>IG_Class</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Class in the SDTMIG v3.4 variable table</t>
+          <t>Target SDTM domain abbreviation (empty for Cross-domain)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SDTMIG_Section</t>
+          <t>Override_Type</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Section number in the SDTMIG v3.4 table of contents</t>
+          <t>Naming (label mismatch), Subset (body-system sub-codelist), or Cross-domain (test code codelist shared by several domains; Domain empty)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Why the dataset is not listed in Domains</t>
+          <t>Description of the mismatch</t>
         </is>
       </c>
     </row>
@@ -995,19 +979,19 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>CONSUMER_EXCLUSIONS COLUMNS</t>
+          <t>INSTRUMENT_DOMAIN_RULES COLUMNS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Consumer</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Findings consumer notebook that reads the row (Specimen_Findings, Measurement_Findings, Instrument_Findings)</t>
+          <t>Instrument class. Matched first as the prefix "CDISC &lt;Keyword&gt; " of the codelist NCI Preferred Term, then as a substring of the codelist display name</t>
         </is>
       </c>
     </row>
@@ -1019,198 +1003,270 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Domain excluded from that consumer's scope</t>
+          <t>Target SDTM domain abbreviation</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Claim_ID</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Identifier of one testable claim behind the exclusion</t>
+          <t>Description and examples of instrument types in this category</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Claim</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>What the published COSMoS content must show for the exclusion reason to hold</t>
-        </is>
-      </c>
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Machine form of the claim, evaluated by domain-behaviour/notebooks/Domain_Behaviour.ipynb: no_fanout, no_axis, not_axis:&lt;axis&gt;, axis_all:&lt;axis&gt;, not_primary:&lt;axis&gt;</t>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>NON_OBSERVATION_DATASETS COLUMNS</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>SDTMIG v3.4 dataset name</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>IG_Name</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Name in the SDTMIG v3.4 table of contents (8.4.1 Supplemental Qualifiers (SUPP--) for SUPPQUAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>IG_Class</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Class in the SDTMIG v3.4 variable table</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>SDTMIG_Section</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Section number in the SDTMIG v3.4 table of contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>The exclusion reason as recorded in the consumer notebook</t>
-        </is>
-      </c>
-    </row>
-    <row r="61"/>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>VARIABLE_MEANING COLUMNS</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Key_Source</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Sheet of domain-behaviour/interim/Domain_Behaviour.xlsx the key must exist in: Variable_Evidence (Domain + variable), Key_Compare (axis; Domain empty), Rater_COSMoS_EVAL (variable_name), Interpretation_Context (Domain + variable, with COSMoS content); or LOINC_Subject_State: sheet Subject_State of cosmos-bc-dss/reports/COSMoS_Observable_LOINC_Check.xlsx (state_variable)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Why the dataset is not listed in Domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>CONSUMER_EXCLUSIONS COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Consumer</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Findings consumer notebook that reads the row (Specimen_Findings, Measurement_Findings, Instrument_Findings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>SDTM domain, Findings class; empty for Key_Compare rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Key</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>The variable, or the axis for Key_Compare rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Position</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>The part of the observable key it identifies: component, system, method, scale; not part of the observable (the published reason in Basis_Note); or open</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>sources agree / sources disagree, decided by a stated rule / standards silent, open</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Basis_Note</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>What each source states, by sheet and column; the rule, where one is used</t>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Domain excluded from that consumer's scope</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>proposed / accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="70"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Identifier of one testable claim behind the exclusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>What the published COSMoS content must show for the exclusion reason to hold</t>
+        </is>
+      </c>
+    </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>KNOWN LIMITATIONS</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="n"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Machine form of the claim, evaluated by domain-behaviour/notebooks/Domain_Behaviour.ipynb: no_fanout, no_axis, not_axis:&lt;axis&gt;, axis_all:&lt;axis&gt;, not_primary:&lt;axis&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Variable-level metadata (key variables, permissible variables) is not included.</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n"/>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>The exclusion reason as recorded in the consumer notebook</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>CDISC publishes it as the SDTM v2.0 and SDTMIG v3.4 variable tables (sign-in at cdisc.org). Local copies sit in sdtm-domain-reference/downloads/ (gitignored); domain-behaviour reads them.</t>
-        </is>
-      </c>
+      <c r="A73" s="2" t="n"/>
       <c r="B73" s="2" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>SDTM v3.0 is under review and may add or change domains.</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="n"/>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>VARIABLE_MEANING COLUMNS</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>MO (Morphology) was decommissioned in v3.4 and is not listed.</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="n"/>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Key_Source</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Sheet of domain-behaviour/interim/Domain_Behaviour.xlsx the key must exist in: Variable_Evidence (Domain + variable), Key_Compare (axis; Domain empty), Rater_COSMoS_EVAL (variable_name), Interpretation_Context (Domain + variable, with COSMoS content); or LOINC_Subject_State: sheet Subject_State of cosmos-bc-dss/reports/COSMoS_Observable_LOINC_Check.xlsx (state_variable)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>SDTMIG_Section, IG_Name, IG_Class, Has_Test_Codes and Specimen_Based, and the Non_Observation_Datasets sheet, are checked against SDTMIG v3.4 by sdtm-findings-graph/notebooks/Scope_Check.ipynb (section 5).</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="n"/>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SDTM domain, Findings class; empty for Key_Compare rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>The variable, or the axis for Key_Compare rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>The part of the observable key it identifies: component, system, method, scale; not part of the observable (the published reason in Basis_Note); or open</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>sources agree / sources disagree, decided by a stated rule / standards silent, open</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Basis_Note</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>What each source states, by sheet and column; the rule, where one is used</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>proposed / accepted</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Domain_Coverage Where_To_Look; 'Not evaluated' flags; domain Notes
Domain_Coverage: new column Where_To_Look, computed from the counts (the
consumer file, else SDTM_Test_Identity / SDTM_Instrument_Test_Identity /
DSS_View, or none); Reason also filled for in-scope domains without DSSs.
SDTM_Domain_Metadata Domains Notes (by hand): PC and PP reasons, BE as
specimen handling events with RELSPEC; Specimen_Findings reads the PC/PP
reasons from there instead of a copy in the notebook.
Findings files: 'Not evaluated' replaces blank in NCIt_Code_Conflict and
NCIt_Reference_Disagree, ReadMe names both causes; Codelists description
says to search synonyms and preferred terms. Landing page: interim files
keep their own ReadMe layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzSyuaqVq1B4PFnRpWB
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -2011,7 +2011,7 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>From SDTMIG-PGx v1.0</t>
+          <t>From SDTMIG-PGx v1.0. Events: specimen handling (collection, culturing, preparation, transport, storage in its COSMoS DSSs). Parent and derived specimens are related in RELSPEC (sheet Non_Observation_Datasets).</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -2893,7 +2893,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>SDTMIG v3.4 binds no codelist to PCTESTCD (the analyte is sponsor-defined), so SDTM_Test_Identity has no PC rows.</t>
+        </is>
+      </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
           <t>Pharmacokinetics Concentrations</t>
@@ -2943,7 +2947,7 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Paired with PC</t>
+          <t>Paired with PC. PPTESTCD is bound to PKPARMCD (C85839), which SDTM_CT_Extract does not read by decision (its section 5b), so SDTM_Test_Identity has no PP rows.</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Variable_Meaning: basis notes cite the IG statements
Basis_Note texts that cited SDTMIG v3.4 assumptions through the interim
IG_Assumptions sheet now cite SDTMIG_Statements.xlsx by Statement_ID
where the text is quoted there (LB-A8, GF-A8, MB-A1a, MB-A1c,
MBTSTDTL-Notes, IS-A8, RS-DR-A1). Ten cells, edited one by one; no
Position, Basis or Status changed.

- VSPOS note corrected: LB Assumption 8 names LBPOS, which is not in the
  SDTMIG v3.4 LB variable table (SDTM v2.0 Findings variable --POS).
- GFMETHOD note: GF Assumption 8 quoted verbatim.
- Rows that only restate the IG (LBSPEC, LBMETHOD, ISBDAGNT, MBTSTDTL)
  stay: the observable key is built from them.
- Findings consumers re-run: Axis_Meaning carries the new notes.
- Docs: Changes_2026-10 paragraph; landing page names Variable_Meaning.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CcwgzTn2VP52uZq6xGb3v7
</commit_message>
<xml_diff>
--- a/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
+++ b/sdtm-domain-reference/machine_actionable/SDTM_Domain_Metadata.xlsx
@@ -5593,7 +5593,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>COSMoS: predicate IS_SPECIMEN_TESTED_IN, "is the specimen tested in", codelist SPECTYPE. Fan-out axis specimen and key part system agree (Key_Compare). LOINC system agrees (LOINC_Compare); the exceptions are COSMoS pin errors reported by COSMoS_Observable_LOINC_Check. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'.</t>
+          <t>COSMoS: predicate IS_SPECIMEN_TESTED_IN, "is the specimen tested in", codelist SPECTYPE. Fan-out axis specimen and key part system agree (Key_Compare). LOINC system agrees (LOINC_Compare); the exceptions are COSMoS pin errors reported by COSMoS_Observable_LOINC_Check. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8: with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'. Quoted in SDTMIG_Statements.xlsx: LB-A8.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>COSMoS: predicate SPECIFIES, "is the method for the test in", DEC Test Method, codelist METHOD. Fan-out axis method and key part method agree (Key_Compare). LOINC method agrees where COSMoS separates by method (LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'.</t>
+          <t>COSMoS: predicate SPECIFIES, "is the method for the test in", DEC Test Method, codelist METHOD. Fan-out axis method and key part method agree (Key_Compare). LOINC method agrees where COSMoS separates by method (LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 LB Assumption 8: with LBTEST and LBORRESU, 'the aspects of a test that are associated with a LOINC code'. Quoted in SDTMIG_Statements.xlsx: LB-A8.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5741,7 +5741,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>COSMoS only: predicate SPECIFIES, DEC Test Method, codelist METHOD. Fan-out and key agree (Key_Compare). GF DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 GF Assumption 8 (IG_Assumptions): 'GFMETHOD lists wet lab techniques …; methods related to specimen processing or reagents are not represented in GFMETHOD.'</t>
+          <t>COSMoS only: predicate SPECIFIES, DEC Test Method, codelist METHOD. Fan-out and key agree (Key_Compare). GF DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, the same role as --POS and --FAST; the role does not separate them. SDTMIG v3.4 GF Assumption 8: 'GFMETHOD lists wet lab techniques for the execution of genomics or genetic testing. Methods related to specimen processing or reagents are not represented in GFMETHOD.' Quoted in SDTMIG_Statements.xlsx: GF-A8.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate SPECIFIES, "further describes the test in", DEC Measurement, Test or Examination Detail, codelist MBFTSDTL. Fan-out and key agree (Key_Compare). LOINC not read for MB (not in LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 MB Assumption 1 (IG_Assumptions): 'DETECTION' for tests that identify an organism; for a characteristic, 'the name of the characteristic being described (e.g., COLONY COUNT, VIRAL LOAD)'.</t>
+          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate SPECIFIES, "further describes the test in", DEC Measurement, Test or Examination Detail, codelist MBFTSDTL. Fan-out and key agree (Key_Compare). LOINC not read for MB (not in LOINC_Compare). SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 MB Assumption 1a, 1c: 'DETECTION' for tests that identify an organism; for a characteristic, 'the name of the characteristic being described (e.g., COLONY COUNT, VIRAL LOAD)'. Quoted in SDTMIG_Statements.xlsx: MB-A1a, MB-A1c, MBTSTDTL-Notes.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate IS_ATTRIBUTE_FOR, "is the substance bound to the analyte in", codelists ISBDAGT and MICROORG. Fan-out axis binding agent and key part component agree (Key_Compare). IS DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 IS Assumption 7 (IG_Assumptions): two codelists (MICROORG, ISBDAGT); the CT Rules for Immunogenicity Tests say which to use. SDTMIG v3.4 CDISC Notes and SDTM v2.0 --BDAGNT: 'the combination of ISTEST and ISBDAGNT should describe the entity or the analyte being measured, without the need for additional variables'; 'not a method qualifier'. Assumption 7a: for antidrug antibody tests the binding agent is the study therapy name, not controlled by CDISC; sponsors extend ISBDAGT. Quoted in SDTMIG_Statements.xlsx: ISBDAGNT-Notes, IS-A7, IS-A7a, IS-A7b.</t>
+          <t>COSMoS and SDTM v2.0/SDTMIG v3.4: predicate IS_ATTRIBUTE_FOR, "is the substance bound to the analyte in", codelists ISBDAGT and MICROORG. Fan-out axis binding agent and key part component agree (Key_Compare). IS DSSs pin no LOINC codes. SDTM v2.0 and SDTMIG v3.4: Variable Qualifier of --TESTCD. SDTMIG v3.4 IS Assumption 7: two codelists (MICROORG, ISBDAGT); the CT Rules for Immunogenicity Tests say which to use. SDTMIG v3.4 CDISC Notes and SDTM v2.0 --BDAGNT: 'the combination of ISTEST and ISBDAGNT should describe the entity or the analyte being measured, without the need for additional variables'; 'not a method qualifier'. Assumption 7a: for antidrug antibody tests the binding agent is the study therapy name, not controlled by CDISC; sponsors extend ISBDAGT. Quoted in SDTMIG_Statements.xlsx: ISBDAGNT-Notes, IS-A7, IS-A7a, IS-A7b.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>COSMoS: value list only (TSTOPOBJ), never assigned; on 64 DSSs in 2 BCs (C187786, C198280). There the DSSs come in 32 pairs with the same binding agent: SCREEN;CONFIRM with result POSITIVE;NEGATIVE and no units (DS code ending PN), QUANTIFY with units. So in COSMoS the tier goes with the scale, which the scale row already separates. SDTMIG v3.4: Variable Qualifier; IS Assumption 8, nonextensible codelist SCREEN, CONFIRM, QUANTIFY; IS Example 1 uses it for the tiers of ADA testing, 'to provide uniqueness to each row of record'. Two readings: the tier is part of the observable, or it is the operational step that produces an observable already told apart by scale. No source says which.</t>
+          <t>COSMoS: value list only (TSTOPOBJ), never assigned; on 64 DSSs in 2 BCs (C187786, C198280). There the DSSs come in 32 pairs with the same binding agent: SCREEN;CONFIRM with result POSITIVE;NEGATIVE and no units (DS code ending PN), QUANTIFY with units. So in COSMoS the tier goes with the scale, which the scale row already separates. SDTMIG v3.4: Variable Qualifier; IS Assumption 8, nonextensible codelist SCREEN, CONFIRM, QUANTIFY; IS Example 1 uses it for the tiers of ADA testing, 'to provide uniqueness to each row of record'. Two readings: the tier is part of the observable, or it is the operational step that produces an observable already told apart by scale. No source says which. Quoted in SDTMIG_Statements.xlsx: IS-A8.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>COSMoS: predicate SPECIFIES, "is the method of secondary analysis of results in", DEC Analysis Method, codelist GFANMET. Not DEC Test Method, so not the test method; the key reads --METHOD only (Key_Compare: method, fan-out only). No source says whether the analysis method is part of the observable. SDTMIG v3.4: Record Qualifier, 'the method of secondary processing performed by the dry lab to yield the result'. SDTMIG v3.4 GF Assumption 8 (IG_Assumptions) confines GFMETHOD to wet lab techniques; the IG note puts GFANMETH in the dry lab (secondary processing).</t>
+          <t>COSMoS: predicate SPECIFIES, "is the method of secondary analysis of results in", DEC Analysis Method, codelist GFANMET. Not DEC Test Method, so not the test method; the key reads --METHOD only (Key_Compare: method, fan-out only). No source says whether the analysis method is part of the observable. SDTMIG v3.4: Record Qualifier, 'the method of secondary processing performed by the dry lab to yield the result'. SDTMIG v3.4 GF Assumption 8 confines GFMETHOD to wet lab techniques; the IG note puts GFANMETH in the dry lab (secondary processing). Quoted in SDTMIG_Statements.xlsx: GF-A8.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>COSMoS: predicate GROUPS, "groups values in", the same as LBCAT. SDTM CT codelist ONCRSCAT, Category of Oncology Response Assessment: the response criteria. Not in the key. No source says whether category changes the observation. SDTM v2.0 and SDTMIG v3.4: Grouping Qualifier; the IG notes that the RSCAT codelist depends on whether the records are oncology response criteria or another clinical classification. SDTMIG v3.4 RS Assumptions (IG_Assumptions; disease response 1, 6, 9; clinical classifications 2): RSCAT 'is used to group a set of assessments based on' a disease response criterion or a clinical classification; 'UNSPECIFIED' when the criteria are unknown.</t>
+          <t>COSMoS: predicate GROUPS, "groups values in", the same as LBCAT. SDTM CT codelist ONCRSCAT, Category of Oncology Response Assessment: the response criteria. Not in the key. No source says whether category changes the observation. SDTM v2.0 and SDTMIG v3.4: Grouping Qualifier; the IG notes that the RSCAT codelist depends on whether the records are oncology response criteria or another clinical classification. SDTMIG v3.4 RS Assumptions (IG_Assumptions; disease response 1, 6, 9; clinical classifications 2): RSCAT 'is used to group a set of assessments based on' a disease response criterion or a clinical classification; 'UNSPECIFIED' when the criteria are unknown. Disease response 1 quoted in SDTMIG_Statements.xlsx: RS-DR-A1.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable. LOINC (Subject_State in COSMoS_Observable_LOINC_Check): position-free and position-qualified codes side by side (^sitting, ^standing, ^supine); COSMoS assigns VSPOS on no DSS. LOINC offers position as a refinement, not as a requirement. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. The SDTMIG v3.4 VS Assumptions do not discuss VSPOS; LB Assumption 8 (IG_Assumptions) names LBPOS (in LB) among the LOINC-associated aspects of a test.</t>
+          <t>COSMoS: predicate IS_SUBJECT_STATE_FOR, "is the subject position during performance of the test in", codelist POSITION. Value list only. COSMoS calls it subject state; no source says whether subject state is part of the observable. LOINC (Subject_State in COSMoS_Observable_LOINC_Check): position-free and position-qualified codes side by side (^sitting, ^standing, ^supine); COSMoS assigns VSPOS on no DSS. LOINC offers position as a refinement, not as a requirement. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. The SDTMIG v3.4 VS Assumptions do not discuss VSPOS; LB Assumption 8 names LBPOS among the LOINC-associated aspects of a test; LBPOS is not in the SDTMIG v3.4 LB variable table (it is the SDTM v2.0 Findings variable --POS). Quoted in SDTMIG_Statements.xlsx: LB-A8.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -6439,7 +6439,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>COSMoS: LBFAST is a value list (N;Y), never assigned, so it never separates sibling DSSs and is not in Variable_Evidence. LOINC (Subject_State): fasting-free and fasting-qualified glucose codes side by side (component Glucose^post CFst, class CHAL). LOINC offers fasting as a refinement, not as a requirement; no source says whether fasting is part of the observable. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. SDTMIG v3.4 LB Assumption 8 (IG_Assumptions): LBFAST is among 'the aspects of a test that are associated with a LOINC code', 'only required to be populated when necessary to provide a semantically meaningful distinction between records with different LBLOINC values'. COSMoS, LOINC and the IG agree that subject state is an optional refinement; none says it is always or never part of the observable (decided 2026-10-08: open, the conditional reading carried into Phase 2).</t>
+          <t>COSMoS: LBFAST is a value list (N;Y), never assigned, so it never separates sibling DSSs and is not in Variable_Evidence. LOINC (Subject_State): fasting-free and fasting-qualified glucose codes side by side (component Glucose^post CFst, class CHAL). LOINC offers fasting as a refinement, not as a requirement; no source says whether fasting is part of the observable. SDTM v2.0 and SDTMIG v3.4: Record Qualifier, like --SPEC and --METHOD; no published role separates subject state from identifying qualifiers. SDTMIG v3.4 LB Assumption 8: LBFAST is among 'the aspects of a test that are associated with a LOINC code', 'only required to be populated when necessary to provide a semantically meaningful distinction between records with different LBLOINC values'. COSMoS, LOINC and the IG agree that subject state is an optional refinement; none says it is always or never part of the observable (decided 2026-10-08: open, the conditional reading carried into Phase 2). Quoted in SDTMIG_Statements.xlsx: LB-A8.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">

</xml_diff>